<commit_message>
cleaning-up code and notebook
</commit_message>
<xml_diff>
--- a/coding/output/output_cycle.xlsx
+++ b/coding/output/output_cycle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkb\Documents\GitHub\Modellierungsseminar-Firestation\coding\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{420C34AA-FF21-40E8-9122-59BACA14E885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB8ACD9-6678-4A23-8ED5-C7184003A47F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FBFD2000-7869-4467-9A00-A335B650FC49}"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11295" xr2:uid="{FBFD2000-7869-4467-9A00-A335B650FC49}"/>
   </bookViews>
   <sheets>
     <sheet name="output_cycle" sheetId="1" r:id="rId1"/>
@@ -610,28 +610,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill>
@@ -656,14 +635,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1634,14 +1620,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A4:G21">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="[00day">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="[freeDay_:-)_]">
+      <formula>NOT(ISERROR(SEARCH("[freeDay_:-)_]",A4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="[night">
+      <formula>NOT(ISERROR(SEARCH("[night",A4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="[00day">
       <formula>NOT(ISERROR(SEARCH("[00day",A4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="[night">
-      <formula>NOT(ISERROR(SEARCH("[night",A4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="[freeDay_:-)_]">
-      <formula>NOT(ISERROR(SEARCH("[freeDay_:-)_]",A4)))</formula>
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="reserveShift">
+      <formula>NOT(ISERROR(SEARCH("reserveShift",A4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>